<commit_message>
Menu de Medidores y ajuste para desplegar anios en el formulario
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{276DDB81-CE0E-4C3F-8E2D-5A7718621EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0BFA16B-7389-42CC-8487-355E941CF3B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15504" yWindow="3432" windowWidth="7536" windowHeight="9072" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Criterios de aceptación'!$A$5:$F$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Historias!$A$5:$P$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tareas!$A$5:$J$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tareas!$A$5:$J$257</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Criterios de aceptación'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">Historias!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">Tareas!$5:$5</definedName>
@@ -196,75 +196,75 @@
     <t>Modelo: revisar Activo_Medidor — columnas, FK e índices. Confirmar el índice único del código dentro del cliente.</t>
   </si>
   <si>
+    <t>T-2019</t>
+  </si>
+  <si>
+    <t>SP SEL_ACTIVO_MEDIDOR: listado con filtros opcionales (id, texto, habilitado) y ORDER BY estable. Un solo SP sirve a la grilla y a la ficha.</t>
+  </si>
+  <si>
+    <t>T-2020</t>
+  </si>
+  <si>
+    <t>SP INS_ACTIVO_MEDIDOR: alta dentro de transacción. Valida código único por cliente y sella la fecha con FNC_PAIS_HORA.</t>
+  </si>
+  <si>
+    <t>T-2021</t>
+  </si>
+  <si>
+    <t>SP UPD_ACTIVO_MEDIDOR: edición. Los campos que la ficha no muestra se conservan con ISNULL(@X, columna) para no borrarlos al guardar.</t>
+  </si>
+  <si>
+    <t>T-2022</t>
+  </si>
+  <si>
+    <t>SP DEL_ACTIVO_MEDIDOR: baja lógica. Rechaza con mensaje si el registro tiene dependientes en vez de dejar huérfanos.</t>
+  </si>
+  <si>
+    <t>T-2023</t>
+  </si>
+  <si>
+    <t>Datos de prueba en Activo_Medidor para poder ejercitar los criterios de aceptación.</t>
+  </si>
+  <si>
+    <t>T-2028</t>
+  </si>
+  <si>
+    <t>Listado ActivoMedidors.aspx: grilla con búsqueda, filtro de habilitados y botón Nuevo.</t>
+  </si>
+  <si>
+    <t>T-2029</t>
+  </si>
+  <si>
+    <t>Ficha ActivoMedidor.aspx en RadWindow con las clases sigma-modal-*: campos, validadores y Guardar/Cerrar.</t>
+  </si>
+  <si>
+    <t>T-2030</t>
+  </si>
+  <si>
+    <t>T-2031</t>
+  </si>
+  <si>
+    <t>T-2032</t>
+  </si>
+  <si>
+    <t>T-2033</t>
+  </si>
+  <si>
+    <t>T-2034</t>
+  </si>
+  <si>
+    <t>HU-150</t>
+  </si>
+  <si>
+    <t>Sincronizar los datos hacia el dispositivo</t>
+  </si>
+  <si>
+    <t>Modelo: CREAR la tabla Sincronizacion_Lote — todavía no existe. Columnas, PK, FK a sus padres y columna sin_uuid con índice UNIQUE para que la sincronización no duplique.</t>
+  </si>
+  <si>
     <t>Bryan Chávez</t>
   </si>
   <si>
-    <t>T-2019</t>
-  </si>
-  <si>
-    <t>SP SEL_ACTIVO_MEDIDOR: listado con filtros opcionales (id, texto, habilitado) y ORDER BY estable. Un solo SP sirve a la grilla y a la ficha.</t>
-  </si>
-  <si>
-    <t>T-2020</t>
-  </si>
-  <si>
-    <t>SP INS_ACTIVO_MEDIDOR: alta dentro de transacción. Valida código único por cliente y sella la fecha con FNC_PAIS_HORA.</t>
-  </si>
-  <si>
-    <t>T-2021</t>
-  </si>
-  <si>
-    <t>SP UPD_ACTIVO_MEDIDOR: edición. Los campos que la ficha no muestra se conservan con ISNULL(@X, columna) para no borrarlos al guardar.</t>
-  </si>
-  <si>
-    <t>T-2022</t>
-  </si>
-  <si>
-    <t>SP DEL_ACTIVO_MEDIDOR: baja lógica. Rechaza con mensaje si el registro tiene dependientes en vez de dejar huérfanos.</t>
-  </si>
-  <si>
-    <t>T-2023</t>
-  </si>
-  <si>
-    <t>Datos de prueba en Activo_Medidor para poder ejercitar los criterios de aceptación.</t>
-  </si>
-  <si>
-    <t>T-2028</t>
-  </si>
-  <si>
-    <t>Listado ActivoMedidors.aspx: grilla con búsqueda, filtro de habilitados y botón Nuevo.</t>
-  </si>
-  <si>
-    <t>T-2029</t>
-  </si>
-  <si>
-    <t>Ficha ActivoMedidor.aspx en RadWindow con las clases sigma-modal-*: campos, validadores y Guardar/Cerrar.</t>
-  </si>
-  <si>
-    <t>T-2030</t>
-  </si>
-  <si>
-    <t>T-2031</t>
-  </si>
-  <si>
-    <t>T-2032</t>
-  </si>
-  <si>
-    <t>T-2033</t>
-  </si>
-  <si>
-    <t>T-2034</t>
-  </si>
-  <si>
-    <t>HU-150</t>
-  </si>
-  <si>
-    <t>Sincronizar los datos hacia el dispositivo</t>
-  </si>
-  <si>
-    <t>Modelo: CREAR la tabla Sincronizacion_Lote — todavía no existe. Columnas, PK, FK a sus padres y columna sin_uuid con índice UNIQUE para que la sincronización no duplique.</t>
-  </si>
-  <si>
     <t>T-2035</t>
   </si>
   <si>
@@ -1756,6 +1756,9 @@
     <t>HU-033, HU-032</t>
   </si>
   <si>
+    <t>En curso</t>
+  </si>
+  <si>
     <t>registrar el horómetro o contador de un equipo</t>
   </si>
   <si>
@@ -1895,9 +1898,6 @@
   </si>
   <si>
     <t>recuperar el servicio sin depender de una gestión telefonica</t>
-  </si>
-  <si>
-    <t>En curso</t>
   </si>
   <si>
     <t>Construida el 02-09-2026 por Bryan Chávez: INS y SEL_SUSCRIPCION_PAGO del bloque 41, Pago.aspx y Pagos.aspx, comprobante como Archivo categoria 12. La correccion se construyo el 02-09 (bloque 59, UPD_SUSCRIPCION_PAGO). FALTAN los datos de prueba: el script esta listo pero no hay periodos emitidos sobre los que sembrar (T-2212). Y la verificacion de los criterios, que es de Catalina.</t>
@@ -3304,7 +3304,7 @@
         <v>528</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
@@ -3514,10 +3514,10 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B11:H13"/>
+    <mergeCell ref="C21:H21"/>
     <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C16:H16"/>
     <mergeCell ref="C19:H19"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="C21:H21"/>
     <mergeCell ref="C22:H22"/>
     <mergeCell ref="B43:H44"/>
     <mergeCell ref="C23:H23"/>
@@ -3693,7 +3693,7 @@
         <v>9.25</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>43</v>
+        <v>574</v>
       </c>
       <c r="O6" s="12"/>
       <c r="P6" s="12"/>
@@ -3712,10 +3712,10 @@
         <v>569</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="G7" s="13" t="s">
         <v>31</v>
@@ -3747,25 +3747,25 @@
     </row>
     <row r="8" spans="1:16" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>550</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="H8" s="11">
         <v>13</v>
@@ -3803,16 +3803,16 @@
         <v>103</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="H9" s="13">
         <v>5</v>
@@ -3850,16 +3850,16 @@
         <v>122</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="H10" s="11">
         <v>3</v>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="O10" s="12"/>
       <c r="P10" s="12" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -3899,16 +3899,16 @@
         <v>144</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="H11" s="13">
         <v>5</v>
@@ -3920,7 +3920,7 @@
         <v>572</v>
       </c>
       <c r="K11" s="14" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="L11" s="13">
         <v>4</v>
@@ -3949,10 +3949,10 @@
         <v>569</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>31</v>
@@ -3967,7 +3967,7 @@
         <v>572</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="L12" s="11">
         <v>2</v>
@@ -3996,10 +3996,10 @@
         <v>569</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="G13" s="13" t="s">
         <v>31</v>
@@ -4011,7 +4011,7 @@
         <v>80</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K13" s="14" t="s">
         <v>13</v>
@@ -4040,16 +4040,16 @@
         <v>208</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="H14" s="11">
         <v>5</v>
@@ -4058,7 +4058,7 @@
         <v>80</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K14" s="12" t="s">
         <v>412</v>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="O14" s="12"/>
       <c r="P14" s="12" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -4089,16 +4089,16 @@
         <v>229</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="H15" s="13">
         <v>5</v>
@@ -4107,7 +4107,7 @@
         <v>80</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K15" s="14" t="s">
         <v>279</v>
@@ -4120,13 +4120,13 @@
         <v>7.5</v>
       </c>
       <c r="N15" s="13" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="O15" s="14" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="P15" s="14" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -4140,16 +4140,16 @@
         <v>260</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="H16" s="11">
         <v>3</v>
@@ -4158,7 +4158,7 @@
         <v>75</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K16" s="12" t="s">
         <v>13</v>
@@ -4187,13 +4187,13 @@
         <v>280</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="G17" s="13" t="s">
         <v>31</v>
@@ -4205,7 +4205,7 @@
         <v>75</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K17" s="14" t="s">
         <v>331</v>
@@ -4218,13 +4218,13 @@
         <v>5.75</v>
       </c>
       <c r="N17" s="13" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="O17" s="14" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="P17" s="14" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -4241,10 +4241,10 @@
         <v>569</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="G18" s="11" t="s">
         <v>31</v>
@@ -4256,7 +4256,7 @@
         <v>70</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K18" s="12" t="s">
         <v>165</v>
@@ -4285,13 +4285,13 @@
         <v>319</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>31</v>
@@ -4303,7 +4303,7 @@
         <v>70</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K19" s="14" t="s">
         <v>207</v>
@@ -4332,13 +4332,13 @@
         <v>332</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="G20" s="11" t="s">
         <v>31</v>
@@ -4350,10 +4350,10 @@
         <v>70</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="L20" s="11">
         <v>3</v>
@@ -4363,13 +4363,13 @@
         <v>5.5</v>
       </c>
       <c r="N20" s="11" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="O20" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="P20" s="12" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="69" customHeight="1" x14ac:dyDescent="0.3">
@@ -4383,13 +4383,13 @@
         <v>364</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>31</v>
@@ -4401,7 +4401,7 @@
         <v>70</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K21" s="14" t="s">
         <v>228</v>
@@ -4414,10 +4414,10 @@
         <v>5.75</v>
       </c>
       <c r="N21" s="13" t="s">
-        <v>621</v>
+        <v>574</v>
       </c>
       <c r="O21" s="14" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="P21" s="14" t="s">
         <v>622</v>
@@ -4452,10 +4452,10 @@
         <v>65</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="L22" s="11">
         <v>2</v>
@@ -4499,7 +4499,7 @@
         <v>65</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K23" s="14" t="s">
         <v>469</v>
@@ -4528,7 +4528,7 @@
         <v>435</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E24" s="12" t="s">
         <v>627</v>
@@ -4546,7 +4546,7 @@
         <v>65</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="K24" s="12" t="s">
         <v>279</v>
@@ -4622,7 +4622,7 @@
         <v>470</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E26" s="12" t="s">
         <v>632</v>
@@ -4643,7 +4643,7 @@
         <v>631</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="L26" s="11">
         <v>2</v>
@@ -4775,7 +4775,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J315"/>
@@ -4853,7 +4853,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>12</v>
       </c>
@@ -4881,7 +4881,7 @@
       <c r="I6" s="11"/>
       <c r="J6" s="12"/>
     </row>
-    <row r="7" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>19</v>
       </c>
@@ -4909,7 +4909,7 @@
       <c r="I7" s="11"/>
       <c r="J7" s="12"/>
     </row>
-    <row r="8" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>21</v>
       </c>
@@ -4937,7 +4937,7 @@
       <c r="I8" s="11"/>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>23</v>
       </c>
@@ -4965,7 +4965,7 @@
       <c r="I9" s="11"/>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>25</v>
       </c>
@@ -4993,7 +4993,7 @@
       <c r="I10" s="11"/>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>27</v>
       </c>
@@ -5021,7 +5021,7 @@
       <c r="I11" s="11"/>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>29</v>
       </c>
@@ -5049,7 +5049,7 @@
       <c r="I12" s="11"/>
       <c r="J12" s="12"/>
     </row>
-    <row r="13" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>32</v>
       </c>
@@ -5077,7 +5077,7 @@
       <c r="I13" s="11"/>
       <c r="J13" s="12"/>
     </row>
-    <row r="14" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>34</v>
       </c>
@@ -5105,7 +5105,7 @@
       <c r="I14" s="11"/>
       <c r="J14" s="12"/>
     </row>
-    <row r="15" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>36</v>
       </c>
@@ -5133,7 +5133,7 @@
       <c r="I15" s="11"/>
       <c r="J15" s="12"/>
     </row>
-    <row r="16" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>39</v>
       </c>
@@ -5161,7 +5161,7 @@
       <c r="I16" s="11"/>
       <c r="J16" s="12"/>
     </row>
-    <row r="17" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>44</v>
       </c>
@@ -5189,7 +5189,7 @@
       <c r="I17" s="11"/>
       <c r="J17" s="12"/>
     </row>
-    <row r="18" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>47</v>
       </c>
@@ -5237,17 +5237,17 @@
         <v>0.5</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I19" s="11"/>
       <c r="J19" s="12"/>
     </row>
     <row r="20" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>51</v>
@@ -5256,7 +5256,7 @@
         <v>52</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>16</v>
@@ -5268,14 +5268,14 @@
         <v>17</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I20" s="11"/>
       <c r="J20" s="12"/>
     </row>
     <row r="21" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>51</v>
@@ -5284,7 +5284,7 @@
         <v>52</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>16</v>
@@ -5293,17 +5293,17 @@
         <v>0.25</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I21" s="11"/>
       <c r="J21" s="12"/>
     </row>
     <row r="22" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>51</v>
@@ -5312,7 +5312,7 @@
         <v>52</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>16</v>
@@ -5321,17 +5321,17 @@
         <v>0.25</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I22" s="11"/>
       <c r="J22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>51</v>
@@ -5340,7 +5340,7 @@
         <v>52</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>16</v>
@@ -5352,14 +5352,14 @@
         <v>17</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I23" s="11"/>
       <c r="J23" s="12"/>
     </row>
     <row r="24" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>51</v>
@@ -5368,7 +5368,7 @@
         <v>52</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>16</v>
@@ -5377,17 +5377,17 @@
         <v>0.25</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I24" s="11"/>
       <c r="J24" s="12"/>
     </row>
     <row r="25" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>51</v>
@@ -5396,7 +5396,7 @@
         <v>52</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>31</v>
@@ -5408,14 +5408,14 @@
         <v>17</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I25" s="11"/>
       <c r="J25" s="12"/>
     </row>
     <row r="26" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>51</v>
@@ -5424,7 +5424,7 @@
         <v>52</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>31</v>
@@ -5433,17 +5433,17 @@
         <v>0.25</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I26" s="11"/>
       <c r="J26" s="12"/>
     </row>
     <row r="27" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>51</v>
@@ -5464,14 +5464,14 @@
         <v>17</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I27" s="11"/>
       <c r="J27" s="12"/>
     </row>
     <row r="28" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>51</v>
@@ -5492,14 +5492,14 @@
         <v>17</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I28" s="11"/>
       <c r="J28" s="12"/>
     </row>
-    <row r="29" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>51</v>
@@ -5525,9 +5525,9 @@
       <c r="I29" s="11"/>
       <c r="J29" s="12"/>
     </row>
-    <row r="30" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>51</v>
@@ -5553,18 +5553,18 @@
       <c r="I30" s="11"/>
       <c r="J30" s="12"/>
     </row>
-    <row r="31" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="C31" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="D31" s="17" t="s">
         <v>75</v>
-      </c>
-      <c r="D31" s="17" t="s">
-        <v>76</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>16</v>
@@ -5573,7 +5573,7 @@
         <v>1.5</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H31" s="11" t="s">
         <v>43</v>
@@ -5581,15 +5581,15 @@
       <c r="I31" s="11"/>
       <c r="J31" s="12"/>
     </row>
-    <row r="32" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
         <v>77</v>
       </c>
       <c r="B32" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D32" s="17" t="s">
         <v>78</v>
@@ -5609,15 +5609,15 @@
       <c r="I32" s="11"/>
       <c r="J32" s="12"/>
     </row>
-    <row r="33" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
         <v>79</v>
       </c>
       <c r="B33" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D33" s="17" t="s">
         <v>80</v>
@@ -5637,15 +5637,15 @@
       <c r="I33" s="11"/>
       <c r="J33" s="12"/>
     </row>
-    <row r="34" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
         <v>81</v>
       </c>
       <c r="B34" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D34" s="17" t="s">
         <v>82</v>
@@ -5657,7 +5657,7 @@
         <v>1.25</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H34" s="11" t="s">
         <v>43</v>
@@ -5665,15 +5665,15 @@
       <c r="I34" s="11"/>
       <c r="J34" s="12"/>
     </row>
-    <row r="35" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
         <v>83</v>
       </c>
       <c r="B35" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D35" s="17" t="s">
         <v>84</v>
@@ -5685,7 +5685,7 @@
         <v>1.5</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H35" s="11" t="s">
         <v>43</v>
@@ -5693,15 +5693,15 @@
       <c r="I35" s="11"/>
       <c r="J35" s="12"/>
     </row>
-    <row r="36" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>86</v>
       </c>
       <c r="B36" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D36" s="17" t="s">
         <v>87</v>
@@ -5721,15 +5721,15 @@
       <c r="I36" s="11"/>
       <c r="J36" s="12"/>
     </row>
-    <row r="37" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
         <v>88</v>
       </c>
       <c r="B37" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D37" s="17" t="s">
         <v>89</v>
@@ -5741,7 +5741,7 @@
         <v>1.25</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H37" s="11" t="s">
         <v>43</v>
@@ -5749,15 +5749,15 @@
       <c r="I37" s="11"/>
       <c r="J37" s="12"/>
     </row>
-    <row r="38" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
         <v>90</v>
       </c>
       <c r="B38" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C38" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D38" s="17" t="s">
         <v>91</v>
@@ -5769,7 +5769,7 @@
         <v>0.75</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H38" s="11" t="s">
         <v>43</v>
@@ -5777,15 +5777,15 @@
       <c r="I38" s="11"/>
       <c r="J38" s="12"/>
     </row>
-    <row r="39" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
         <v>93</v>
       </c>
       <c r="B39" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C39" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C39" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D39" s="17" t="s">
         <v>94</v>
@@ -5805,15 +5805,15 @@
       <c r="I39" s="11"/>
       <c r="J39" s="12"/>
     </row>
-    <row r="40" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
         <v>95</v>
       </c>
       <c r="B40" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C40" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D40" s="17" t="s">
         <v>96</v>
@@ -5825,7 +5825,7 @@
         <v>0.75</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H40" s="11" t="s">
         <v>43</v>
@@ -5833,15 +5833,15 @@
       <c r="I40" s="11"/>
       <c r="J40" s="12"/>
     </row>
-    <row r="41" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
         <v>97</v>
       </c>
       <c r="B41" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C41" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D41" s="17" t="s">
         <v>37</v>
@@ -5853,7 +5853,7 @@
         <v>1.5</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H41" s="11" t="s">
         <v>43</v>
@@ -5861,15 +5861,15 @@
       <c r="I41" s="11"/>
       <c r="J41" s="12"/>
     </row>
-    <row r="42" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="11" t="s">
         <v>98</v>
       </c>
       <c r="B42" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C42" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C42" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D42" s="17" t="s">
         <v>40</v>
@@ -5889,15 +5889,15 @@
       <c r="I42" s="11"/>
       <c r="J42" s="12"/>
     </row>
-    <row r="43" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="11" t="s">
         <v>99</v>
       </c>
       <c r="B43" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C43" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D43" s="17" t="s">
         <v>45</v>
@@ -5917,15 +5917,15 @@
       <c r="I43" s="11"/>
       <c r="J43" s="12"/>
     </row>
-    <row r="44" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
         <v>100</v>
       </c>
       <c r="B44" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C44" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="C44" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>48</v>
@@ -6021,7 +6021,7 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H47" s="11" t="s">
         <v>43</v>
@@ -6105,7 +6105,7 @@
         <v>0.75</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H50" s="11" t="s">
         <v>43</v>
@@ -6141,7 +6141,7 @@
       <c r="I51" s="11"/>
       <c r="J51" s="12"/>
     </row>
-    <row r="52" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="11" t="s">
         <v>115</v>
       </c>
@@ -6197,7 +6197,7 @@
       <c r="I53" s="11"/>
       <c r="J53" s="12"/>
     </row>
-    <row r="54" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="11" t="s">
         <v>118</v>
       </c>
@@ -6225,7 +6225,7 @@
       <c r="I54" s="11"/>
       <c r="J54" s="12"/>
     </row>
-    <row r="55" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="11" t="s">
         <v>119</v>
       </c>
@@ -6253,7 +6253,7 @@
       <c r="I55" s="11"/>
       <c r="J55" s="12"/>
     </row>
-    <row r="56" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="11" t="s">
         <v>120</v>
       </c>
@@ -6281,7 +6281,7 @@
       <c r="I56" s="11"/>
       <c r="J56" s="12"/>
     </row>
-    <row r="57" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
         <v>124</v>
       </c>
@@ -6301,7 +6301,7 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H57" s="11" t="s">
         <v>43</v>
@@ -6309,7 +6309,7 @@
       <c r="I57" s="11"/>
       <c r="J57" s="12"/>
     </row>
-    <row r="58" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="11" t="s">
         <v>126</v>
       </c>
@@ -6337,7 +6337,7 @@
       <c r="I58" s="11"/>
       <c r="J58" s="12"/>
     </row>
-    <row r="59" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="11" t="s">
         <v>128</v>
       </c>
@@ -6365,7 +6365,7 @@
       <c r="I59" s="11"/>
       <c r="J59" s="12"/>
     </row>
-    <row r="60" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="11" t="s">
         <v>130</v>
       </c>
@@ -6385,7 +6385,7 @@
         <v>0.25</v>
       </c>
       <c r="G60" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H60" s="11" t="s">
         <v>43</v>
@@ -6393,7 +6393,7 @@
       <c r="I60" s="11"/>
       <c r="J60" s="12"/>
     </row>
-    <row r="61" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="11" t="s">
         <v>132</v>
       </c>
@@ -6421,7 +6421,7 @@
       <c r="I61" s="11"/>
       <c r="J61" s="12"/>
     </row>
-    <row r="62" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="11" t="s">
         <v>134</v>
       </c>
@@ -6441,7 +6441,7 @@
         <v>0.25</v>
       </c>
       <c r="G62" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H62" s="11" t="s">
         <v>43</v>
@@ -6449,7 +6449,7 @@
       <c r="I62" s="11"/>
       <c r="J62" s="12"/>
     </row>
-    <row r="63" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="11" t="s">
         <v>136</v>
       </c>
@@ -6477,7 +6477,7 @@
       <c r="I63" s="11"/>
       <c r="J63" s="12"/>
     </row>
-    <row r="64" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="11" t="s">
         <v>138</v>
       </c>
@@ -6497,7 +6497,7 @@
         <v>0.25</v>
       </c>
       <c r="G64" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H64" s="11" t="s">
         <v>43</v>
@@ -6505,7 +6505,7 @@
       <c r="I64" s="11"/>
       <c r="J64" s="12"/>
     </row>
-    <row r="65" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="11" t="s">
         <v>139</v>
       </c>
@@ -6525,7 +6525,7 @@
         <v>0.25</v>
       </c>
       <c r="G65" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H65" s="11" t="s">
         <v>43</v>
@@ -6533,7 +6533,7 @@
       <c r="I65" s="11"/>
       <c r="J65" s="12"/>
     </row>
-    <row r="66" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="11" t="s">
         <v>140</v>
       </c>
@@ -6561,7 +6561,7 @@
       <c r="I66" s="11"/>
       <c r="J66" s="12"/>
     </row>
-    <row r="67" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="11" t="s">
         <v>141</v>
       </c>
@@ -6589,7 +6589,7 @@
       <c r="I67" s="11"/>
       <c r="J67" s="12"/>
     </row>
-    <row r="68" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="11" t="s">
         <v>142</v>
       </c>
@@ -6617,7 +6617,7 @@
       <c r="I68" s="11"/>
       <c r="J68" s="12"/>
     </row>
-    <row r="69" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="11" t="s">
         <v>146</v>
       </c>
@@ -6645,7 +6645,7 @@
       <c r="I69" s="11"/>
       <c r="J69" s="12"/>
     </row>
-    <row r="70" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="11" t="s">
         <v>148</v>
       </c>
@@ -6665,7 +6665,7 @@
         <v>0.5</v>
       </c>
       <c r="G70" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H70" s="11" t="s">
         <v>43</v>
@@ -6673,7 +6673,7 @@
       <c r="I70" s="11"/>
       <c r="J70" s="12"/>
     </row>
-    <row r="71" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="11" t="s">
         <v>150</v>
       </c>
@@ -6701,7 +6701,7 @@
       <c r="I71" s="11"/>
       <c r="J71" s="12"/>
     </row>
-    <row r="72" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="11" t="s">
         <v>152</v>
       </c>
@@ -6721,7 +6721,7 @@
         <v>0.75</v>
       </c>
       <c r="G72" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H72" s="11" t="s">
         <v>43</v>
@@ -6729,7 +6729,7 @@
       <c r="I72" s="11"/>
       <c r="J72" s="12"/>
     </row>
-    <row r="73" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="11" t="s">
         <v>154</v>
       </c>
@@ -6757,7 +6757,7 @@
       <c r="I73" s="11"/>
       <c r="J73" s="12"/>
     </row>
-    <row r="74" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="11" t="s">
         <v>156</v>
       </c>
@@ -6777,7 +6777,7 @@
         <v>0.5</v>
       </c>
       <c r="G74" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H74" s="11" t="s">
         <v>43</v>
@@ -6785,7 +6785,7 @@
       <c r="I74" s="11"/>
       <c r="J74" s="12"/>
     </row>
-    <row r="75" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="11" t="s">
         <v>157</v>
       </c>
@@ -6813,7 +6813,7 @@
       <c r="I75" s="11"/>
       <c r="J75" s="12"/>
     </row>
-    <row r="76" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="11" t="s">
         <v>159</v>
       </c>
@@ -6833,7 +6833,7 @@
         <v>0.25</v>
       </c>
       <c r="G76" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H76" s="11" t="s">
         <v>43</v>
@@ -6841,7 +6841,7 @@
       <c r="I76" s="11"/>
       <c r="J76" s="12"/>
     </row>
-    <row r="77" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="11" t="s">
         <v>160</v>
       </c>
@@ -6869,7 +6869,7 @@
       <c r="I77" s="11"/>
       <c r="J77" s="12"/>
     </row>
-    <row r="78" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="11" t="s">
         <v>161</v>
       </c>
@@ -6897,7 +6897,7 @@
       <c r="I78" s="11"/>
       <c r="J78" s="12"/>
     </row>
-    <row r="79" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="11" t="s">
         <v>162</v>
       </c>
@@ -6925,7 +6925,7 @@
       <c r="I79" s="11"/>
       <c r="J79" s="12"/>
     </row>
-    <row r="80" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="11" t="s">
         <v>163</v>
       </c>
@@ -6953,7 +6953,7 @@
       <c r="I80" s="11"/>
       <c r="J80" s="12"/>
     </row>
-    <row r="81" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="11" t="s">
         <v>164</v>
       </c>
@@ -6981,7 +6981,7 @@
       <c r="I81" s="11"/>
       <c r="J81" s="12"/>
     </row>
-    <row r="82" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="11" t="s">
         <v>167</v>
       </c>
@@ -7001,7 +7001,7 @@
         <v>0.5</v>
       </c>
       <c r="G82" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H82" s="11" t="s">
         <v>43</v>
@@ -7009,7 +7009,7 @@
       <c r="I82" s="11"/>
       <c r="J82" s="12"/>
     </row>
-    <row r="83" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="11" t="s">
         <v>169</v>
       </c>
@@ -7037,7 +7037,7 @@
       <c r="I83" s="11"/>
       <c r="J83" s="12"/>
     </row>
-    <row r="84" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="11" t="s">
         <v>171</v>
       </c>
@@ -7065,7 +7065,7 @@
       <c r="I84" s="11"/>
       <c r="J84" s="12"/>
     </row>
-    <row r="85" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="11" t="s">
         <v>173</v>
       </c>
@@ -7085,7 +7085,7 @@
         <v>0.5</v>
       </c>
       <c r="G85" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H85" s="11" t="s">
         <v>43</v>
@@ -7093,7 +7093,7 @@
       <c r="I85" s="11"/>
       <c r="J85" s="12"/>
     </row>
-    <row r="86" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="11" t="s">
         <v>175</v>
       </c>
@@ -7121,7 +7121,7 @@
       <c r="I86" s="11"/>
       <c r="J86" s="12"/>
     </row>
-    <row r="87" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="11" t="s">
         <v>176</v>
       </c>
@@ -7149,7 +7149,7 @@
       <c r="I87" s="11"/>
       <c r="J87" s="12"/>
     </row>
-    <row r="88" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="11" t="s">
         <v>178</v>
       </c>
@@ -7169,7 +7169,7 @@
         <v>0.5</v>
       </c>
       <c r="G88" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H88" s="11" t="s">
         <v>43</v>
@@ -7177,7 +7177,7 @@
       <c r="I88" s="11"/>
       <c r="J88" s="12"/>
     </row>
-    <row r="89" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="11" t="s">
         <v>180</v>
       </c>
@@ -7205,7 +7205,7 @@
       <c r="I89" s="11"/>
       <c r="J89" s="12"/>
     </row>
-    <row r="90" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="11" t="s">
         <v>181</v>
       </c>
@@ -7225,7 +7225,7 @@
         <v>0.5</v>
       </c>
       <c r="G90" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H90" s="11" t="s">
         <v>43</v>
@@ -7233,7 +7233,7 @@
       <c r="I90" s="11"/>
       <c r="J90" s="12"/>
     </row>
-    <row r="91" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="11" t="s">
         <v>182</v>
       </c>
@@ -7261,7 +7261,7 @@
       <c r="I91" s="11"/>
       <c r="J91" s="12"/>
     </row>
-    <row r="92" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="11" t="s">
         <v>183</v>
       </c>
@@ -7337,7 +7337,7 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H94" s="11" t="s">
         <v>43</v>
@@ -7421,7 +7421,7 @@
         <v>0.5</v>
       </c>
       <c r="G97" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H97" s="11" t="s">
         <v>43</v>
@@ -7477,7 +7477,7 @@
         <v>0.5</v>
       </c>
       <c r="G99" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H99" s="11" t="s">
         <v>43</v>
@@ -7533,7 +7533,7 @@
         <v>0.5</v>
       </c>
       <c r="G101" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H101" s="11" t="s">
         <v>43</v>
@@ -7569,7 +7569,7 @@
       <c r="I102" s="11"/>
       <c r="J102" s="12"/>
     </row>
-    <row r="103" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="11" t="s">
         <v>204</v>
       </c>
@@ -7597,7 +7597,7 @@
       <c r="I103" s="11"/>
       <c r="J103" s="12"/>
     </row>
-    <row r="104" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="11" t="s">
         <v>205</v>
       </c>
@@ -7625,7 +7625,7 @@
       <c r="I104" s="11"/>
       <c r="J104" s="12"/>
     </row>
-    <row r="105" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="11" t="s">
         <v>206</v>
       </c>
@@ -7653,7 +7653,7 @@
       <c r="I105" s="11"/>
       <c r="J105" s="12"/>
     </row>
-    <row r="106" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="11" t="s">
         <v>210</v>
       </c>
@@ -7673,7 +7673,7 @@
         <v>0.5</v>
       </c>
       <c r="G106" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H106" s="11" t="s">
         <v>43</v>
@@ -7681,7 +7681,7 @@
       <c r="I106" s="11"/>
       <c r="J106" s="12"/>
     </row>
-    <row r="107" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="11" t="s">
         <v>212</v>
       </c>
@@ -7709,7 +7709,7 @@
       <c r="I107" s="11"/>
       <c r="J107" s="12"/>
     </row>
-    <row r="108" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="11" t="s">
         <v>214</v>
       </c>
@@ -7737,7 +7737,7 @@
       <c r="I108" s="11"/>
       <c r="J108" s="12"/>
     </row>
-    <row r="109" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="11" t="s">
         <v>216</v>
       </c>
@@ -7757,7 +7757,7 @@
         <v>0.5</v>
       </c>
       <c r="G109" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H109" s="11" t="s">
         <v>43</v>
@@ -7765,7 +7765,7 @@
       <c r="I109" s="11"/>
       <c r="J109" s="12"/>
     </row>
-    <row r="110" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="11" t="s">
         <v>218</v>
       </c>
@@ -7793,7 +7793,7 @@
       <c r="I110" s="11"/>
       <c r="J110" s="12"/>
     </row>
-    <row r="111" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="11" t="s">
         <v>220</v>
       </c>
@@ -7813,7 +7813,7 @@
         <v>0.5</v>
       </c>
       <c r="G111" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H111" s="11" t="s">
         <v>43</v>
@@ -7821,7 +7821,7 @@
       <c r="I111" s="11"/>
       <c r="J111" s="12"/>
     </row>
-    <row r="112" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="11" t="s">
         <v>222</v>
       </c>
@@ -7849,7 +7849,7 @@
       <c r="I112" s="11"/>
       <c r="J112" s="12"/>
     </row>
-    <row r="113" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="11" t="s">
         <v>223</v>
       </c>
@@ -7869,7 +7869,7 @@
         <v>0.5</v>
       </c>
       <c r="G113" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H113" s="11" t="s">
         <v>43</v>
@@ -7877,7 +7877,7 @@
       <c r="I113" s="11"/>
       <c r="J113" s="12"/>
     </row>
-    <row r="114" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="11" t="s">
         <v>224</v>
       </c>
@@ -7897,7 +7897,7 @@
         <v>0.5</v>
       </c>
       <c r="G114" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H114" s="11" t="s">
         <v>43</v>
@@ -7905,7 +7905,7 @@
       <c r="I114" s="11"/>
       <c r="J114" s="12"/>
     </row>
-    <row r="115" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="11" t="s">
         <v>225</v>
       </c>
@@ -7933,7 +7933,7 @@
       <c r="I115" s="11"/>
       <c r="J115" s="12"/>
     </row>
-    <row r="116" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="11" t="s">
         <v>226</v>
       </c>
@@ -7961,7 +7961,7 @@
       <c r="I116" s="11"/>
       <c r="J116" s="12"/>
     </row>
-    <row r="117" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="11" t="s">
         <v>227</v>
       </c>
@@ -7981,7 +7981,7 @@
         <v>0.5</v>
       </c>
       <c r="G117" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H117" s="11" t="s">
         <v>18</v>
@@ -7993,7 +7993,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="118" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="11" t="s">
         <v>232</v>
       </c>
@@ -8013,7 +8013,7 @@
         <v>0.5</v>
       </c>
       <c r="G118" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H118" s="11" t="s">
         <v>18</v>
@@ -8025,7 +8025,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="11" t="s">
         <v>235</v>
       </c>
@@ -8045,7 +8045,7 @@
         <v>0.5</v>
       </c>
       <c r="G119" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H119" s="11" t="s">
         <v>18</v>
@@ -8057,7 +8057,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="11" t="s">
         <v>238</v>
       </c>
@@ -8077,7 +8077,7 @@
         <v>0.5</v>
       </c>
       <c r="G120" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H120" s="11" t="s">
         <v>18</v>
@@ -8089,7 +8089,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="11" t="s">
         <v>241</v>
       </c>
@@ -8109,7 +8109,7 @@
         <v>0.5</v>
       </c>
       <c r="G121" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H121" s="11" t="s">
         <v>18</v>
@@ -8121,7 +8121,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="11" t="s">
         <v>244</v>
       </c>
@@ -8141,7 +8141,7 @@
         <v>0.75</v>
       </c>
       <c r="G122" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H122" s="11" t="s">
         <v>18</v>
@@ -8153,7 +8153,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="123" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="11" t="s">
         <v>247</v>
       </c>
@@ -8173,7 +8173,7 @@
         <v>0.75</v>
       </c>
       <c r="G123" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H123" s="11" t="s">
         <v>18</v>
@@ -8185,7 +8185,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="11" t="s">
         <v>250</v>
       </c>
@@ -8205,7 +8205,7 @@
         <v>1.25</v>
       </c>
       <c r="G124" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H124" s="11" t="s">
         <v>18</v>
@@ -8217,7 +8217,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="125" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="11" t="s">
         <v>253</v>
       </c>
@@ -8245,7 +8245,7 @@
       <c r="I125" s="11"/>
       <c r="J125" s="12"/>
     </row>
-    <row r="126" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="11" t="s">
         <v>254</v>
       </c>
@@ -8265,7 +8265,7 @@
         <v>0.5</v>
       </c>
       <c r="G126" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H126" s="11" t="s">
         <v>18</v>
@@ -8277,7 +8277,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="127" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="11" t="s">
         <v>256</v>
       </c>
@@ -8305,7 +8305,7 @@
       <c r="I127" s="11"/>
       <c r="J127" s="12"/>
     </row>
-    <row r="128" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="11" t="s">
         <v>257</v>
       </c>
@@ -8353,7 +8353,7 @@
         <v>0.5</v>
       </c>
       <c r="G129" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H129" s="11" t="s">
         <v>43</v>
@@ -8437,7 +8437,7 @@
         <v>0.25</v>
       </c>
       <c r="G132" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H132" s="11" t="s">
         <v>43</v>
@@ -8493,7 +8493,7 @@
         <v>0.5</v>
       </c>
       <c r="G134" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H134" s="11" t="s">
         <v>43</v>
@@ -8549,7 +8549,7 @@
         <v>0.75</v>
       </c>
       <c r="G136" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H136" s="11" t="s">
         <v>43</v>
@@ -8557,7 +8557,7 @@
       <c r="I136" s="11"/>
       <c r="J136" s="12"/>
     </row>
-    <row r="137" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="11" t="s">
         <v>274</v>
       </c>
@@ -8577,7 +8577,7 @@
         <v>0.25</v>
       </c>
       <c r="G137" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H137" s="11" t="s">
         <v>43</v>
@@ -8605,7 +8605,7 @@
         <v>0.25</v>
       </c>
       <c r="G138" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H138" s="11" t="s">
         <v>43</v>
@@ -8613,7 +8613,7 @@
       <c r="I138" s="11"/>
       <c r="J138" s="12"/>
     </row>
-    <row r="139" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="11" t="s">
         <v>276</v>
       </c>
@@ -8641,7 +8641,7 @@
       <c r="I139" s="11"/>
       <c r="J139" s="12"/>
     </row>
-    <row r="140" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="11" t="s">
         <v>277</v>
       </c>
@@ -8669,7 +8669,7 @@
       <c r="I140" s="11"/>
       <c r="J140" s="12"/>
     </row>
-    <row r="141" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="11" t="s">
         <v>278</v>
       </c>
@@ -8689,7 +8689,7 @@
         <v>0.75</v>
       </c>
       <c r="G141" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H141" s="11" t="s">
         <v>18</v>
@@ -8701,7 +8701,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="142" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="11" t="s">
         <v>282</v>
       </c>
@@ -8721,7 +8721,7 @@
         <v>0.5</v>
       </c>
       <c r="G142" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H142" s="11" t="s">
         <v>18</v>
@@ -8733,7 +8733,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="143" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="11" t="s">
         <v>285</v>
       </c>
@@ -8753,7 +8753,7 @@
         <v>0.5</v>
       </c>
       <c r="G143" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H143" s="11" t="s">
         <v>18</v>
@@ -8765,7 +8765,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="144" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="11" t="s">
         <v>288</v>
       </c>
@@ -8785,7 +8785,7 @@
         <v>0.5</v>
       </c>
       <c r="G144" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H144" s="11" t="s">
         <v>18</v>
@@ -8797,7 +8797,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="11" t="s">
         <v>291</v>
       </c>
@@ -8817,7 +8817,7 @@
         <v>0.5</v>
       </c>
       <c r="G145" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H145" s="11" t="s">
         <v>18</v>
@@ -8829,7 +8829,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="11" t="s">
         <v>293</v>
       </c>
@@ -8849,7 +8849,7 @@
         <v>0.75</v>
       </c>
       <c r="G146" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H146" s="11" t="s">
         <v>18</v>
@@ -8861,7 +8861,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="151.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:10" ht="151.80000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="11" t="s">
         <v>296</v>
       </c>
@@ -8881,7 +8881,7 @@
         <v>0.75</v>
       </c>
       <c r="G147" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H147" s="11" t="s">
         <v>18</v>
@@ -8893,7 +8893,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="11" t="s">
         <v>299</v>
       </c>
@@ -8913,7 +8913,7 @@
         <v>0.5</v>
       </c>
       <c r="G148" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H148" s="11" t="s">
         <v>18</v>
@@ -8925,7 +8925,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="11" t="s">
         <v>301</v>
       </c>
@@ -8953,7 +8953,7 @@
       <c r="I149" s="11"/>
       <c r="J149" s="12"/>
     </row>
-    <row r="150" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="11" t="s">
         <v>302</v>
       </c>
@@ -8981,7 +8981,7 @@
       <c r="I150" s="11"/>
       <c r="J150" s="12"/>
     </row>
-    <row r="151" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="11" t="s">
         <v>303</v>
       </c>
@@ -9009,7 +9009,7 @@
       <c r="I151" s="11"/>
       <c r="J151" s="12"/>
     </row>
-    <row r="152" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="11" t="s">
         <v>306</v>
       </c>
@@ -9037,7 +9037,7 @@
       <c r="I152" s="11"/>
       <c r="J152" s="12"/>
     </row>
-    <row r="153" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="11" t="s">
         <v>308</v>
       </c>
@@ -9057,7 +9057,7 @@
         <v>0.5</v>
       </c>
       <c r="G153" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H153" s="11" t="s">
         <v>43</v>
@@ -9065,7 +9065,7 @@
       <c r="I153" s="11"/>
       <c r="J153" s="12"/>
     </row>
-    <row r="154" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="11" t="s">
         <v>309</v>
       </c>
@@ -9093,7 +9093,7 @@
       <c r="I154" s="11"/>
       <c r="J154" s="12"/>
     </row>
-    <row r="155" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="11" t="s">
         <v>311</v>
       </c>
@@ -9121,7 +9121,7 @@
       <c r="I155" s="11"/>
       <c r="J155" s="12"/>
     </row>
-    <row r="156" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="11" t="s">
         <v>312</v>
       </c>
@@ -9149,7 +9149,7 @@
       <c r="I156" s="11"/>
       <c r="J156" s="12"/>
     </row>
-    <row r="157" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="11" t="s">
         <v>314</v>
       </c>
@@ -9169,7 +9169,7 @@
         <v>0.25</v>
       </c>
       <c r="G157" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H157" s="11" t="s">
         <v>43</v>
@@ -9177,7 +9177,7 @@
       <c r="I157" s="11"/>
       <c r="J157" s="12"/>
     </row>
-    <row r="158" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="11" t="s">
         <v>315</v>
       </c>
@@ -9205,7 +9205,7 @@
       <c r="I158" s="11"/>
       <c r="J158" s="12"/>
     </row>
-    <row r="159" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="11" t="s">
         <v>316</v>
       </c>
@@ -9233,7 +9233,7 @@
       <c r="I159" s="11"/>
       <c r="J159" s="12"/>
     </row>
-    <row r="160" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="11" t="s">
         <v>317</v>
       </c>
@@ -9253,7 +9253,7 @@
         <v>0.75</v>
       </c>
       <c r="G160" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H160" s="11" t="s">
         <v>43</v>
@@ -9261,7 +9261,7 @@
       <c r="I160" s="11"/>
       <c r="J160" s="12"/>
     </row>
-    <row r="161" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="11" t="s">
         <v>320</v>
       </c>
@@ -9289,7 +9289,7 @@
       <c r="I161" s="11"/>
       <c r="J161" s="12"/>
     </row>
-    <row r="162" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="11" t="s">
         <v>322</v>
       </c>
@@ -9317,7 +9317,7 @@
       <c r="I162" s="11"/>
       <c r="J162" s="12"/>
     </row>
-    <row r="163" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="11" t="s">
         <v>324</v>
       </c>
@@ -9337,7 +9337,7 @@
         <v>0.5</v>
       </c>
       <c r="G163" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H163" s="11" t="s">
         <v>43</v>
@@ -9345,7 +9345,7 @@
       <c r="I163" s="11"/>
       <c r="J163" s="12"/>
     </row>
-    <row r="164" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="11" t="s">
         <v>325</v>
       </c>
@@ -9365,7 +9365,7 @@
         <v>1.5</v>
       </c>
       <c r="G164" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H164" s="11" t="s">
         <v>43</v>
@@ -9373,7 +9373,7 @@
       <c r="I164" s="11"/>
       <c r="J164" s="12"/>
     </row>
-    <row r="165" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="11" t="s">
         <v>327</v>
       </c>
@@ -9401,7 +9401,7 @@
       <c r="I165" s="11"/>
       <c r="J165" s="12"/>
     </row>
-    <row r="166" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="11" t="s">
         <v>328</v>
       </c>
@@ -9429,7 +9429,7 @@
       <c r="I166" s="11"/>
       <c r="J166" s="12"/>
     </row>
-    <row r="167" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="11" t="s">
         <v>329</v>
       </c>
@@ -9457,7 +9457,7 @@
       <c r="I167" s="11"/>
       <c r="J167" s="12"/>
     </row>
-    <row r="168" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="11" t="s">
         <v>330</v>
       </c>
@@ -9477,7 +9477,7 @@
         <v>0.5</v>
       </c>
       <c r="G168" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H168" s="11" t="s">
         <v>18</v>
@@ -9489,7 +9489,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="169" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="11" t="s">
         <v>335</v>
       </c>
@@ -9509,7 +9509,7 @@
         <v>0.5</v>
       </c>
       <c r="G169" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H169" s="11" t="s">
         <v>18</v>
@@ -9521,7 +9521,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="11" t="s">
         <v>338</v>
       </c>
@@ -9541,7 +9541,7 @@
         <v>0.5</v>
       </c>
       <c r="G170" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H170" s="11" t="s">
         <v>18</v>
@@ -9553,7 +9553,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="171" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="11" t="s">
         <v>341</v>
       </c>
@@ -9573,7 +9573,7 @@
         <v>0.5</v>
       </c>
       <c r="G171" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H171" s="11" t="s">
         <v>18</v>
@@ -9585,7 +9585,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="11" t="s">
         <v>344</v>
       </c>
@@ -9605,7 +9605,7 @@
         <v>0.5</v>
       </c>
       <c r="G172" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H172" s="11" t="s">
         <v>18</v>
@@ -9617,7 +9617,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="173" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="11" t="s">
         <v>347</v>
       </c>
@@ -9637,7 +9637,7 @@
         <v>0.25</v>
       </c>
       <c r="G173" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H173" s="11" t="s">
         <v>18</v>
@@ -9649,7 +9649,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="174" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="11" t="s">
         <v>350</v>
       </c>
@@ -9669,7 +9669,7 @@
         <v>0.5</v>
       </c>
       <c r="G174" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H174" s="11" t="s">
         <v>18</v>
@@ -9681,7 +9681,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="175" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="11" t="s">
         <v>353</v>
       </c>
@@ -9701,7 +9701,7 @@
         <v>0.5</v>
       </c>
       <c r="G175" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H175" s="11" t="s">
         <v>18</v>
@@ -9713,7 +9713,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="176" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="11" t="s">
         <v>356</v>
       </c>
@@ -9733,7 +9733,7 @@
         <v>0.5</v>
       </c>
       <c r="G176" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H176" s="11" t="s">
         <v>18</v>
@@ -9745,7 +9745,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="177" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="11" t="s">
         <v>358</v>
       </c>
@@ -9765,7 +9765,7 @@
         <v>0.5</v>
       </c>
       <c r="G177" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H177" s="11" t="s">
         <v>18</v>
@@ -9777,7 +9777,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="178" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="11" t="s">
         <v>360</v>
       </c>
@@ -9805,7 +9805,7 @@
       <c r="I178" s="11"/>
       <c r="J178" s="12"/>
     </row>
-    <row r="179" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="11" t="s">
         <v>361</v>
       </c>
@@ -9833,7 +9833,7 @@
       <c r="I179" s="11"/>
       <c r="J179" s="12"/>
     </row>
-    <row r="180" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="11" t="s">
         <v>362</v>
       </c>
@@ -9853,7 +9853,7 @@
         <v>0.75</v>
       </c>
       <c r="G180" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H180" s="11" t="s">
         <v>18</v>
@@ -9865,7 +9865,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="181" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="11" t="s">
         <v>367</v>
       </c>
@@ -9885,7 +9885,7 @@
         <v>0.5</v>
       </c>
       <c r="G181" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H181" s="11" t="s">
         <v>18</v>
@@ -9897,7 +9897,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="182" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="11" t="s">
         <v>370</v>
       </c>
@@ -9917,7 +9917,7 @@
         <v>0.5</v>
       </c>
       <c r="G182" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H182" s="11" t="s">
         <v>18</v>
@@ -9929,7 +9929,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="183" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="11" t="s">
         <v>373</v>
       </c>
@@ -9949,7 +9949,7 @@
         <v>0.5</v>
       </c>
       <c r="G183" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H183" s="11" t="s">
         <v>18</v>
@@ -9961,7 +9961,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="184" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="11" t="s">
         <v>376</v>
       </c>
@@ -9981,7 +9981,7 @@
         <v>0.5</v>
       </c>
       <c r="G184" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H184" s="11" t="s">
         <v>43</v>
@@ -9991,7 +9991,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="185" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="11" t="s">
         <v>379</v>
       </c>
@@ -10011,7 +10011,7 @@
         <v>0.75</v>
       </c>
       <c r="G185" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H185" s="11" t="s">
         <v>18</v>
@@ -10023,7 +10023,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="186" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="11" t="s">
         <v>382</v>
       </c>
@@ -10043,7 +10043,7 @@
         <v>0.75</v>
       </c>
       <c r="G186" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H186" s="11" t="s">
         <v>18</v>
@@ -10055,7 +10055,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="187" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="11" t="s">
         <v>385</v>
       </c>
@@ -10075,7 +10075,7 @@
         <v>0.5</v>
       </c>
       <c r="G187" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H187" s="11" t="s">
         <v>18</v>
@@ -10087,7 +10087,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="188" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="11" t="s">
         <v>387</v>
       </c>
@@ -10115,7 +10115,7 @@
       <c r="I188" s="11"/>
       <c r="J188" s="12"/>
     </row>
-    <row r="189" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="11" t="s">
         <v>388</v>
       </c>
@@ -10163,7 +10163,7 @@
         <v>0.5</v>
       </c>
       <c r="G190" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H190" s="11" t="s">
         <v>43</v>
@@ -10247,7 +10247,7 @@
         <v>0.5</v>
       </c>
       <c r="G193" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H193" s="11" t="s">
         <v>43</v>
@@ -10331,7 +10331,7 @@
         <v>0.5</v>
       </c>
       <c r="G196" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H196" s="11" t="s">
         <v>43</v>
@@ -10387,7 +10387,7 @@
         <v>0.5</v>
       </c>
       <c r="G198" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H198" s="11" t="s">
         <v>43</v>
@@ -10415,7 +10415,7 @@
         <v>0.5</v>
       </c>
       <c r="G199" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H199" s="11" t="s">
         <v>43</v>
@@ -10423,7 +10423,7 @@
       <c r="I199" s="11"/>
       <c r="J199" s="12"/>
     </row>
-    <row r="200" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="11" t="s">
         <v>409</v>
       </c>
@@ -10451,7 +10451,7 @@
       <c r="I200" s="11"/>
       <c r="J200" s="12"/>
     </row>
-    <row r="201" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="11" t="s">
         <v>410</v>
       </c>
@@ -10479,7 +10479,7 @@
       <c r="I201" s="11"/>
       <c r="J201" s="12"/>
     </row>
-    <row r="202" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A202" s="11" t="s">
         <v>411</v>
       </c>
@@ -10499,7 +10499,7 @@
         <v>0.5</v>
       </c>
       <c r="G202" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H202" s="11" t="s">
         <v>43</v>
@@ -10507,7 +10507,7 @@
       <c r="I202" s="11"/>
       <c r="J202" s="12"/>
     </row>
-    <row r="203" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A203" s="11" t="s">
         <v>415</v>
       </c>
@@ -10535,7 +10535,7 @@
       <c r="I203" s="11"/>
       <c r="J203" s="12"/>
     </row>
-    <row r="204" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A204" s="11" t="s">
         <v>417</v>
       </c>
@@ -10563,7 +10563,7 @@
       <c r="I204" s="11"/>
       <c r="J204" s="12"/>
     </row>
-    <row r="205" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A205" s="11" t="s">
         <v>419</v>
       </c>
@@ -10583,7 +10583,7 @@
         <v>0.5</v>
       </c>
       <c r="G205" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H205" s="11" t="s">
         <v>43</v>
@@ -10591,7 +10591,7 @@
       <c r="I205" s="11"/>
       <c r="J205" s="12"/>
     </row>
-    <row r="206" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A206" s="11" t="s">
         <v>421</v>
       </c>
@@ -10619,7 +10619,7 @@
       <c r="I206" s="11"/>
       <c r="J206" s="12"/>
     </row>
-    <row r="207" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A207" s="11" t="s">
         <v>423</v>
       </c>
@@ -10647,7 +10647,7 @@
       <c r="I207" s="11"/>
       <c r="J207" s="12"/>
     </row>
-    <row r="208" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A208" s="11" t="s">
         <v>425</v>
       </c>
@@ -10675,7 +10675,7 @@
       <c r="I208" s="11"/>
       <c r="J208" s="12"/>
     </row>
-    <row r="209" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A209" s="11" t="s">
         <v>427</v>
       </c>
@@ -10695,7 +10695,7 @@
         <v>0.5</v>
       </c>
       <c r="G209" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H209" s="11" t="s">
         <v>43</v>
@@ -10703,7 +10703,7 @@
       <c r="I209" s="11"/>
       <c r="J209" s="12"/>
     </row>
-    <row r="210" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A210" s="11" t="s">
         <v>429</v>
       </c>
@@ -10731,7 +10731,7 @@
       <c r="I210" s="11"/>
       <c r="J210" s="12"/>
     </row>
-    <row r="211" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A211" s="11" t="s">
         <v>430</v>
       </c>
@@ -10759,7 +10759,7 @@
       <c r="I211" s="11"/>
       <c r="J211" s="12"/>
     </row>
-    <row r="212" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A212" s="11" t="s">
         <v>431</v>
       </c>
@@ -10787,7 +10787,7 @@
       <c r="I212" s="11"/>
       <c r="J212" s="12"/>
     </row>
-    <row r="213" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A213" s="11" t="s">
         <v>432</v>
       </c>
@@ -10815,7 +10815,7 @@
       <c r="I213" s="11"/>
       <c r="J213" s="12"/>
     </row>
-    <row r="214" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="11" t="s">
         <v>433</v>
       </c>
@@ -10835,7 +10835,7 @@
         <v>0.5</v>
       </c>
       <c r="G214" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H214" s="11" t="s">
         <v>43</v>
@@ -10843,7 +10843,7 @@
       <c r="I214" s="11"/>
       <c r="J214" s="12"/>
     </row>
-    <row r="215" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A215" s="11" t="s">
         <v>436</v>
       </c>
@@ -10871,7 +10871,7 @@
       <c r="I215" s="11"/>
       <c r="J215" s="12"/>
     </row>
-    <row r="216" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A216" s="11" t="s">
         <v>438</v>
       </c>
@@ -10899,7 +10899,7 @@
       <c r="I216" s="11"/>
       <c r="J216" s="12"/>
     </row>
-    <row r="217" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A217" s="11" t="s">
         <v>440</v>
       </c>
@@ -10919,7 +10919,7 @@
         <v>0.25</v>
       </c>
       <c r="G217" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H217" s="11" t="s">
         <v>43</v>
@@ -10927,7 +10927,7 @@
       <c r="I217" s="11"/>
       <c r="J217" s="12"/>
     </row>
-    <row r="218" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A218" s="11" t="s">
         <v>441</v>
       </c>
@@ -10947,7 +10947,7 @@
         <v>0.75</v>
       </c>
       <c r="G218" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H218" s="11" t="s">
         <v>43</v>
@@ -10955,7 +10955,7 @@
       <c r="I218" s="11"/>
       <c r="J218" s="12"/>
     </row>
-    <row r="219" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A219" s="11" t="s">
         <v>443</v>
       </c>
@@ -10975,7 +10975,7 @@
         <v>0.25</v>
       </c>
       <c r="G219" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H219" s="11" t="s">
         <v>43</v>
@@ -10983,7 +10983,7 @@
       <c r="I219" s="11"/>
       <c r="J219" s="12"/>
     </row>
-    <row r="220" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A220" s="11" t="s">
         <v>444</v>
       </c>
@@ -11011,7 +11011,7 @@
       <c r="I220" s="11"/>
       <c r="J220" s="12"/>
     </row>
-    <row r="221" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A221" s="11" t="s">
         <v>445</v>
       </c>
@@ -11115,7 +11115,7 @@
         <v>0.25</v>
       </c>
       <c r="G224" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H224" s="11" t="s">
         <v>43</v>
@@ -11199,7 +11199,7 @@
         <v>0.25</v>
       </c>
       <c r="G227" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H227" s="11" t="s">
         <v>43</v>
@@ -11255,7 +11255,7 @@
         <v>0.25</v>
       </c>
       <c r="G229" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H229" s="11" t="s">
         <v>43</v>
@@ -11319,7 +11319,7 @@
       <c r="I231" s="11"/>
       <c r="J231" s="12"/>
     </row>
-    <row r="232" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A232" s="11" t="s">
         <v>466</v>
       </c>
@@ -11347,7 +11347,7 @@
       <c r="I232" s="11"/>
       <c r="J232" s="12"/>
     </row>
-    <row r="233" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A233" s="11" t="s">
         <v>467</v>
       </c>
@@ -11375,7 +11375,7 @@
       <c r="I233" s="11"/>
       <c r="J233" s="12"/>
     </row>
-    <row r="234" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A234" s="11" t="s">
         <v>468</v>
       </c>
@@ -11403,7 +11403,7 @@
       <c r="I234" s="11"/>
       <c r="J234" s="12"/>
     </row>
-    <row r="235" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A235" s="11" t="s">
         <v>472</v>
       </c>
@@ -11431,7 +11431,7 @@
       <c r="I235" s="11"/>
       <c r="J235" s="12"/>
     </row>
-    <row r="236" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A236" s="11" t="s">
         <v>474</v>
       </c>
@@ -11451,7 +11451,7 @@
         <v>0.5</v>
       </c>
       <c r="G236" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H236" s="11" t="s">
         <v>43</v>
@@ -11459,7 +11459,7 @@
       <c r="I236" s="11"/>
       <c r="J236" s="12"/>
     </row>
-    <row r="237" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A237" s="11" t="s">
         <v>476</v>
       </c>
@@ -11487,7 +11487,7 @@
       <c r="I237" s="11"/>
       <c r="J237" s="12"/>
     </row>
-    <row r="238" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A238" s="11" t="s">
         <v>478</v>
       </c>
@@ -11515,7 +11515,7 @@
       <c r="I238" s="11"/>
       <c r="J238" s="12"/>
     </row>
-    <row r="239" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A239" s="11" t="s">
         <v>480</v>
       </c>
@@ -11535,7 +11535,7 @@
         <v>0.25</v>
       </c>
       <c r="G239" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H239" s="11" t="s">
         <v>43</v>
@@ -11543,7 +11543,7 @@
       <c r="I239" s="11"/>
       <c r="J239" s="12"/>
     </row>
-    <row r="240" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A240" s="11" t="s">
         <v>482</v>
       </c>
@@ -11563,7 +11563,7 @@
         <v>0.5</v>
       </c>
       <c r="G240" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H240" s="11" t="s">
         <v>43</v>
@@ -11571,7 +11571,7 @@
       <c r="I240" s="11"/>
       <c r="J240" s="12"/>
     </row>
-    <row r="241" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A241" s="11" t="s">
         <v>484</v>
       </c>
@@ -11599,7 +11599,7 @@
       <c r="I241" s="11"/>
       <c r="J241" s="12"/>
     </row>
-    <row r="242" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A242" s="11" t="s">
         <v>486</v>
       </c>
@@ -11619,7 +11619,7 @@
         <v>0.5</v>
       </c>
       <c r="G242" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H242" s="11" t="s">
         <v>43</v>
@@ -11627,7 +11627,7 @@
       <c r="I242" s="11"/>
       <c r="J242" s="12"/>
     </row>
-    <row r="243" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A243" s="11" t="s">
         <v>487</v>
       </c>
@@ -11647,7 +11647,7 @@
         <v>0.5</v>
       </c>
       <c r="G243" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H243" s="11" t="s">
         <v>43</v>
@@ -11655,7 +11655,7 @@
       <c r="I243" s="11"/>
       <c r="J243" s="12"/>
     </row>
-    <row r="244" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A244" s="11" t="s">
         <v>488</v>
       </c>
@@ -11683,7 +11683,7 @@
       <c r="I244" s="11"/>
       <c r="J244" s="12"/>
     </row>
-    <row r="245" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A245" s="11" t="s">
         <v>489</v>
       </c>
@@ -11787,7 +11787,7 @@
         <v>0.5</v>
       </c>
       <c r="G248" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H248" s="11" t="s">
         <v>43</v>
@@ -11871,7 +11871,7 @@
         <v>0.25</v>
       </c>
       <c r="G251" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H251" s="11" t="s">
         <v>43</v>
@@ -11927,7 +11927,7 @@
         <v>0.5</v>
       </c>
       <c r="G253" s="12" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="H253" s="11" t="s">
         <v>43</v>
@@ -11991,7 +11991,7 @@
       <c r="I255" s="11"/>
       <c r="J255" s="12"/>
     </row>
-    <row r="256" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A256" s="11" t="s">
         <v>510</v>
       </c>
@@ -12019,7 +12019,7 @@
       <c r="I256" s="11"/>
       <c r="J256" s="12"/>
     </row>
-    <row r="257" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A257" s="11" t="s">
         <v>511</v>
       </c>
@@ -12104,7 +12104,33 @@
     <row r="314" ht="41.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="315" ht="41.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A5:J141" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A5:J257" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Administrar modelos de activo"/>
+        <filter val="Administrar tipos de activo"/>
+        <filter val="Cambiar el estado de un activo indicando el motivo"/>
+        <filter val="Configurar el medidor de un activo"/>
+        <filter val="Consultar la ficha y el historial de un activo"/>
+        <filter val="Definir los atributos técnicos de un tipo de activo"/>
+        <filter val="Registrar los componentes de un activo"/>
+        <filter val="Registrar un activo"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="API"/>
+        <filter val="Base de datos"/>
+        <filter val="Seguridad"/>
+        <filter val="Web"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Por hacer"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
@@ -12340,10 +12366,10 @@
     </row>
     <row r="13" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>74</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>75</v>
       </c>
       <c r="C13" s="13">
         <v>1</v>
@@ -12360,10 +12386,10 @@
     </row>
     <row r="14" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="C14" s="11">
         <v>2</v>
@@ -12380,10 +12406,10 @@
     </row>
     <row r="15" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>74</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>75</v>
       </c>
       <c r="C15" s="13">
         <v>3</v>

</xml_diff>

<commit_message>
HU-037 ficha e historial de activo + renumero bloques BD (87-92)
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D82FA00-82BF-44CD-BD23-98FE975E5623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B6CB4F6-39C1-456C-95C2-BD4E2A47C274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15504" yWindow="3432" windowWidth="7536" windowHeight="9072" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint" sheetId="1" r:id="rId1"/>
@@ -3514,10 +3514,10 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B11:H13"/>
+    <mergeCell ref="C21:H21"/>
     <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C16:H16"/>
     <mergeCell ref="C19:H19"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="C21:H21"/>
     <mergeCell ref="C22:H22"/>
     <mergeCell ref="B43:H44"/>
     <mergeCell ref="C23:H23"/>
@@ -5217,7 +5217,7 @@
       <c r="I18" s="11"/>
       <c r="J18" s="12"/>
     </row>
-    <row r="19" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>50</v>
       </c>
@@ -5245,7 +5245,7 @@
       <c r="I19" s="11"/>
       <c r="J19" s="12"/>
     </row>
-    <row r="20" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>54</v>
       </c>
@@ -5273,7 +5273,7 @@
       <c r="I20" s="11"/>
       <c r="J20" s="12"/>
     </row>
-    <row r="21" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>56</v>
       </c>
@@ -5301,7 +5301,7 @@
       <c r="I21" s="11"/>
       <c r="J21" s="12"/>
     </row>
-    <row r="22" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>58</v>
       </c>
@@ -5329,7 +5329,7 @@
       <c r="I22" s="11"/>
       <c r="J22" s="12"/>
     </row>
-    <row r="23" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>60</v>
       </c>
@@ -5357,7 +5357,7 @@
       <c r="I23" s="11"/>
       <c r="J23" s="12"/>
     </row>
-    <row r="24" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>62</v>
       </c>
@@ -5385,7 +5385,7 @@
       <c r="I24" s="11"/>
       <c r="J24" s="12"/>
     </row>
-    <row r="25" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>64</v>
       </c>
@@ -5413,7 +5413,7 @@
       <c r="I25" s="11"/>
       <c r="J25" s="12"/>
     </row>
-    <row r="26" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>66</v>
       </c>
@@ -5441,7 +5441,7 @@
       <c r="I26" s="11"/>
       <c r="J26" s="12"/>
     </row>
-    <row r="27" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>68</v>
       </c>
@@ -5469,7 +5469,7 @@
       <c r="I27" s="11"/>
       <c r="J27" s="12"/>
     </row>
-    <row r="28" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>69</v>
       </c>
@@ -5968,7 +5968,7 @@
         <v>17</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I45" s="11"/>
       <c r="J45" s="12"/>
@@ -5993,10 +5993,10 @@
         <v>0.75</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I46" s="11"/>
       <c r="J46" s="12"/>
@@ -6021,10 +6021,10 @@
         <v>0.5</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I47" s="11"/>
       <c r="J47" s="12"/>
@@ -6052,7 +6052,7 @@
         <v>17</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I48" s="11"/>
       <c r="J48" s="12"/>
@@ -6080,7 +6080,7 @@
         <v>17</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I49" s="11"/>
       <c r="J49" s="12"/>
@@ -6105,10 +6105,10 @@
         <v>0.75</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I50" s="11"/>
       <c r="J50" s="12"/>
@@ -6136,7 +6136,7 @@
         <v>17</v>
       </c>
       <c r="H51" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I51" s="11"/>
       <c r="J51" s="12"/>
@@ -6192,7 +6192,7 @@
         <v>17</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I53" s="11"/>
       <c r="J53" s="12"/>
@@ -10143,7 +10143,7 @@
       <c r="I189" s="11"/>
       <c r="J189" s="12"/>
     </row>
-    <row r="190" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="11" t="s">
         <v>389</v>
       </c>
@@ -10171,7 +10171,7 @@
       <c r="I190" s="11"/>
       <c r="J190" s="12"/>
     </row>
-    <row r="191" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="11" t="s">
         <v>393</v>
       </c>
@@ -10199,7 +10199,7 @@
       <c r="I191" s="11"/>
       <c r="J191" s="12"/>
     </row>
-    <row r="192" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="11" t="s">
         <v>395</v>
       </c>
@@ -10227,7 +10227,7 @@
       <c r="I192" s="11"/>
       <c r="J192" s="12"/>
     </row>
-    <row r="193" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="11" t="s">
         <v>397</v>
       </c>
@@ -10255,7 +10255,7 @@
       <c r="I193" s="11"/>
       <c r="J193" s="12"/>
     </row>
-    <row r="194" spans="1:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:10" ht="55.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="11" t="s">
         <v>399</v>
       </c>
@@ -10283,7 +10283,7 @@
       <c r="I194" s="11"/>
       <c r="J194" s="12"/>
     </row>
-    <row r="195" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="11" t="s">
         <v>401</v>
       </c>
@@ -10311,7 +10311,7 @@
       <c r="I195" s="11"/>
       <c r="J195" s="12"/>
     </row>
-    <row r="196" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="11" t="s">
         <v>403</v>
       </c>
@@ -10339,7 +10339,7 @@
       <c r="I196" s="11"/>
       <c r="J196" s="12"/>
     </row>
-    <row r="197" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:10" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="11" t="s">
         <v>405</v>
       </c>
@@ -10367,7 +10367,7 @@
       <c r="I197" s="11"/>
       <c r="J197" s="12"/>
     </row>
-    <row r="198" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="11" t="s">
         <v>407</v>
       </c>
@@ -10395,7 +10395,7 @@
       <c r="I198" s="11"/>
       <c r="J198" s="12"/>
     </row>
-    <row r="199" spans="1:10" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:10" ht="41.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="11" t="s">
         <v>408</v>
       </c>

</xml_diff>

<commit_message>
Mantenedor de unidades de medida (HU-040)
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B6CB4F6-39C1-456C-95C2-BD4E2A47C274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CDDDEA6-7DD0-422B-A384-C0508F704AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15504" yWindow="3432" windowWidth="7536" windowHeight="9072" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3514,10 +3514,10 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B11:H13"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="C16:H16"/>
     <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="C19:H19"/>
     <mergeCell ref="C22:H22"/>
     <mergeCell ref="B43:H44"/>
     <mergeCell ref="C23:H23"/>
@@ -11398,7 +11398,7 @@
         <v>17</v>
       </c>
       <c r="H234" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I234" s="11"/>
       <c r="J234" s="12"/>
@@ -11423,10 +11423,10 @@
         <v>0.5</v>
       </c>
       <c r="G235" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H235" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I235" s="11"/>
       <c r="J235" s="12"/>
@@ -11451,10 +11451,10 @@
         <v>0.5</v>
       </c>
       <c r="G236" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H236" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I236" s="11"/>
       <c r="J236" s="12"/>
@@ -11482,7 +11482,7 @@
         <v>17</v>
       </c>
       <c r="H237" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I237" s="11"/>
       <c r="J237" s="12"/>
@@ -11507,10 +11507,10 @@
         <v>0.5</v>
       </c>
       <c r="G238" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H238" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I238" s="11"/>
       <c r="J238" s="12"/>
@@ -11535,10 +11535,10 @@
         <v>0.25</v>
       </c>
       <c r="G239" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H239" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I239" s="11"/>
       <c r="J239" s="12"/>
@@ -11563,10 +11563,10 @@
         <v>0.5</v>
       </c>
       <c r="G240" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H240" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I240" s="11"/>
       <c r="J240" s="12"/>
@@ -11594,7 +11594,7 @@
         <v>17</v>
       </c>
       <c r="H241" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I241" s="11"/>
       <c r="J241" s="12"/>
@@ -11619,10 +11619,10 @@
         <v>0.5</v>
       </c>
       <c r="G242" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H242" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I242" s="11"/>
       <c r="J242" s="12"/>
@@ -11647,10 +11647,10 @@
         <v>0.5</v>
       </c>
       <c r="G243" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H243" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I243" s="11"/>
       <c r="J243" s="12"/>

</xml_diff>

<commit_message>
HU-036 componentes de activo y codigo automatico (MED/COM/TIP/UNI)
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CDDDEA6-7DD0-422B-A384-C0508F704AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1600E5EF-322B-489C-AD90-FB3AED775A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15504" yWindow="3432" windowWidth="7536" windowHeight="9072" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint" sheetId="1" r:id="rId1"/>
@@ -7309,10 +7309,10 @@
         <v>0.5</v>
       </c>
       <c r="G93" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H93" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I93" s="11"/>
       <c r="J93" s="12"/>
@@ -7337,10 +7337,10 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H94" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I94" s="11"/>
       <c r="J94" s="12"/>
@@ -7368,7 +7368,7 @@
         <v>17</v>
       </c>
       <c r="H95" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I95" s="11"/>
       <c r="J95" s="12"/>
@@ -7393,10 +7393,10 @@
         <v>0.5</v>
       </c>
       <c r="G96" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H96" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I96" s="11"/>
       <c r="J96" s="12"/>
@@ -7421,10 +7421,10 @@
         <v>0.5</v>
       </c>
       <c r="G97" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H97" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I97" s="11"/>
       <c r="J97" s="12"/>
@@ -7452,7 +7452,7 @@
         <v>17</v>
       </c>
       <c r="H98" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I98" s="11"/>
       <c r="J98" s="12"/>
@@ -7477,10 +7477,10 @@
         <v>0.5</v>
       </c>
       <c r="G99" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H99" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I99" s="11"/>
       <c r="J99" s="12"/>
@@ -7508,7 +7508,7 @@
         <v>17</v>
       </c>
       <c r="H100" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I100" s="11"/>
       <c r="J100" s="12"/>
@@ -7533,10 +7533,10 @@
         <v>0.5</v>
       </c>
       <c r="G101" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H101" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I101" s="11"/>
       <c r="J101" s="12"/>
@@ -7564,7 +7564,7 @@
         <v>17</v>
       </c>
       <c r="H102" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I102" s="11"/>
       <c r="J102" s="12"/>

</xml_diff>

<commit_message>
HU-038 cambio de estado de activo (proceso, web y API)
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1600E5EF-322B-489C-AD90-FB3AED775A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD2546D2-DE23-4961-B0CB-33DCF64FC3C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8353,10 +8353,10 @@
         <v>0.5</v>
       </c>
       <c r="G129" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H129" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I129" s="11"/>
       <c r="J129" s="12"/>
@@ -8384,7 +8384,7 @@
         <v>17</v>
       </c>
       <c r="H130" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I130" s="11"/>
       <c r="J130" s="12"/>
@@ -8409,10 +8409,10 @@
         <v>0.25</v>
       </c>
       <c r="G131" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H131" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I131" s="11"/>
       <c r="J131" s="12"/>
@@ -8437,10 +8437,10 @@
         <v>0.25</v>
       </c>
       <c r="G132" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H132" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I132" s="11"/>
       <c r="J132" s="12"/>
@@ -8468,7 +8468,7 @@
         <v>17</v>
       </c>
       <c r="H133" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I133" s="11"/>
       <c r="J133" s="12"/>
@@ -8493,10 +8493,10 @@
         <v>0.5</v>
       </c>
       <c r="G134" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H134" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I134" s="11"/>
       <c r="J134" s="12"/>
@@ -8524,7 +8524,7 @@
         <v>17</v>
       </c>
       <c r="H135" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I135" s="11"/>
       <c r="J135" s="12"/>
@@ -8549,10 +8549,10 @@
         <v>0.75</v>
       </c>
       <c r="G136" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H136" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I136" s="11"/>
       <c r="J136" s="12"/>
@@ -8605,10 +8605,10 @@
         <v>0.25</v>
       </c>
       <c r="G138" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H138" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I138" s="11"/>
       <c r="J138" s="12"/>

</xml_diff>

<commit_message>
HU-031 administrar modelos de activo
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD2546D2-DE23-4961-B0CB-33DCF64FC3C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732B707F-13BC-492E-AA4B-211E22E77C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2431" uniqueCount="779">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2432" uniqueCount="779">
   <si>
     <t>Sprint 2 · Tareas del Sprint</t>
   </si>
@@ -3514,10 +3514,10 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B11:H13"/>
+    <mergeCell ref="C21:H21"/>
     <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C16:H16"/>
     <mergeCell ref="C19:H19"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="C21:H21"/>
     <mergeCell ref="C22:H22"/>
     <mergeCell ref="B43:H44"/>
     <mergeCell ref="C23:H23"/>
@@ -4653,9 +4653,11 @@
         <v>5.5</v>
       </c>
       <c r="N26" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="O26" s="12"/>
+        <v>18</v>
+      </c>
+      <c r="O26" s="12" t="s">
+        <v>17</v>
+      </c>
       <c r="P26" s="12"/>
     </row>
     <row r="27" spans="1:16" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -11062,7 +11064,7 @@
         <v>17</v>
       </c>
       <c r="H222" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I222" s="11"/>
       <c r="J222" s="12"/>
@@ -11087,10 +11089,10 @@
         <v>0.25</v>
       </c>
       <c r="G223" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H223" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I223" s="11"/>
       <c r="J223" s="12"/>
@@ -11115,10 +11117,10 @@
         <v>0.25</v>
       </c>
       <c r="G224" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H224" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I224" s="11"/>
       <c r="J224" s="12"/>
@@ -11146,7 +11148,7 @@
         <v>17</v>
       </c>
       <c r="H225" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I225" s="11"/>
       <c r="J225" s="12"/>
@@ -11171,10 +11173,10 @@
         <v>0.25</v>
       </c>
       <c r="G226" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H226" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I226" s="11"/>
       <c r="J226" s="12"/>
@@ -11199,10 +11201,10 @@
         <v>0.25</v>
       </c>
       <c r="G227" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H227" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I227" s="11"/>
       <c r="J227" s="12"/>
@@ -11230,7 +11232,7 @@
         <v>17</v>
       </c>
       <c r="H228" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I228" s="11"/>
       <c r="J228" s="12"/>
@@ -11255,10 +11257,10 @@
         <v>0.25</v>
       </c>
       <c r="G229" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H229" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I229" s="11"/>
       <c r="J229" s="12"/>
@@ -11286,7 +11288,7 @@
         <v>17</v>
       </c>
       <c r="H230" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I230" s="11"/>
       <c r="J230" s="12"/>
@@ -11314,7 +11316,7 @@
         <v>17</v>
       </c>
       <c r="H231" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I231" s="11"/>
       <c r="J231" s="12"/>

</xml_diff>

<commit_message>
HU-032 definir atributos tecnicos de tipo de activo
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 2\Sprint Backlogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732B707F-13BC-492E-AA4B-211E22E77C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C93C91B-537B-4296-92D3-F7CCAC41890C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3514,10 +3514,10 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B11:H13"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="C16:H16"/>
     <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="C19:H19"/>
     <mergeCell ref="C22:H22"/>
     <mergeCell ref="B43:H44"/>
     <mergeCell ref="C23:H23"/>
@@ -11736,7 +11736,7 @@
         <v>17</v>
       </c>
       <c r="H246" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I246" s="11"/>
       <c r="J246" s="12"/>
@@ -11761,10 +11761,10 @@
         <v>0.5</v>
       </c>
       <c r="G247" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H247" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I247" s="11"/>
       <c r="J247" s="12"/>
@@ -11789,10 +11789,10 @@
         <v>0.5</v>
       </c>
       <c r="G248" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H248" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I248" s="11"/>
       <c r="J248" s="12"/>
@@ -11820,7 +11820,7 @@
         <v>17</v>
       </c>
       <c r="H249" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I249" s="11"/>
       <c r="J249" s="12"/>
@@ -11845,10 +11845,10 @@
         <v>0.5</v>
       </c>
       <c r="G250" s="12" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="H250" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I250" s="11"/>
       <c r="J250" s="12"/>
@@ -11873,10 +11873,10 @@
         <v>0.25</v>
       </c>
       <c r="G251" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H251" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I251" s="11"/>
       <c r="J251" s="12"/>
@@ -11904,7 +11904,7 @@
         <v>17</v>
       </c>
       <c r="H252" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I252" s="11"/>
       <c r="J252" s="12"/>
@@ -11929,10 +11929,10 @@
         <v>0.5</v>
       </c>
       <c r="G253" s="12" t="s">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="H253" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I253" s="11"/>
       <c r="J253" s="12"/>
@@ -11960,7 +11960,7 @@
         <v>17</v>
       </c>
       <c r="H254" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I254" s="11"/>
       <c r="J254" s="12"/>
@@ -11988,7 +11988,7 @@
         <v>17</v>
       </c>
       <c r="H255" s="11" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="I255" s="11"/>
       <c r="J255" s="12"/>

</xml_diff>